<commit_message>
Cambio de alcance (Sprint Review 1): la app movil se entrega en el Sprint 6
- Actas Scrum del Sprint 1 (Review y Retrospective) en Fase 2/Ceremonias.
- Product Backlog por Sprint: 22 historias App (154 pts) pasan al Sprint 6;
  Sprint 6 renombrado App movil, inteligencia y cierre.
- Sprint Backlogs S1-S5: tareas Movil e historias App quedan Movida a Sprint 6
  y aparecen en S6 con su estado; Web y App en S6 con 0 pts (solo parte movil).
- Burndown: puntos comprometidos por Sprint actualizados.
- Checklist 10.20 y bitacora.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
@@ -3306,11 +3306,15 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Movida a Sprint 6</t>
         </is>
       </c>
       <c r="I14" s="11" t="n"/>
-      <c r="J14" s="20" t="n"/>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>Movida al Sprint 6 (Sprint Review 1, 15-09-2026). Estado al moverla: Por hacer.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="55.15" customHeight="1" s="24">
       <c r="A15" s="11" t="inlineStr">
@@ -3826,11 +3830,15 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Movida a Sprint 6</t>
         </is>
       </c>
       <c r="I26" s="11" t="n"/>
-      <c r="J26" s="20" t="n"/>
+      <c r="J26" s="20" t="inlineStr">
+        <is>
+          <t>Movida al Sprint 6 (Sprint Review 1, 15-09-2026). Estado al moverla: Por hacer.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="41.45" customHeight="1" s="24">
       <c r="A27" s="11" t="inlineStr">
@@ -4178,13 +4186,13 @@
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Movida a Sprint 6</t>
         </is>
       </c>
       <c r="I34" s="11" t="n"/>
       <c r="J34" s="20" t="inlineStr">
         <is>
-          <t>Nace de la correccion de alcance de la app (30-08-2026).</t>
+          <t>Movida al Sprint 6 (Sprint Review 1, 15-09-2026). Estado al moverla: Por hacer. Nace de la correccion de alcance de la app (30-08-2026).</t>
         </is>
       </c>
     </row>
@@ -5310,11 +5318,15 @@
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Movida a Sprint 6</t>
         </is>
       </c>
       <c r="I60" s="11" t="n"/>
-      <c r="J60" s="20" t="n"/>
+      <c r="J60" s="20" t="inlineStr">
+        <is>
+          <t>Movida al Sprint 6 (Sprint Review 1, 15-09-2026). Estado al moverla: Por hacer.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="41.45" customHeight="1" s="24">
       <c r="A61" s="11" t="inlineStr">
@@ -7956,11 +7968,15 @@
       </c>
       <c r="H121" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Movida a Sprint 6</t>
         </is>
       </c>
       <c r="I121" s="11" t="n"/>
-      <c r="J121" s="20" t="n"/>
+      <c r="J121" s="20" t="inlineStr">
+        <is>
+          <t>Movida al Sprint 6 (Sprint Review 1, 15-09-2026). Estado al moverla: Por hacer.</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="41.45" customHeight="1" s="24">
       <c r="A122" s="11" t="inlineStr">
@@ -11382,13 +11398,13 @@
       </c>
       <c r="H200" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Movida a Sprint 6</t>
         </is>
       </c>
       <c r="I200" s="11" t="n"/>
       <c r="J200" s="20" t="inlineStr">
         <is>
-          <t>Nace de la correccion de alcance de la app (30-08-2026).</t>
+          <t>Movida al Sprint 6 (Sprint Review 1, 15-09-2026). Estado al moverla: Por hacer. Nace de la correccion de alcance de la app (30-08-2026).</t>
         </is>
       </c>
     </row>
@@ -13258,11 +13274,15 @@
       </c>
       <c r="H243" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Movida a Sprint 6</t>
         </is>
       </c>
       <c r="I243" s="11" t="n"/>
-      <c r="J243" s="20" t="n"/>
+      <c r="J243" s="20" t="inlineStr">
+        <is>
+          <t>Movida al Sprint 6 (Sprint Review 1, 15-09-2026). Estado al moverla: Por hacer.</t>
+        </is>
+      </c>
     </row>
     <row r="244" ht="27.6" customHeight="1" s="24">
       <c r="A244" s="11" t="inlineStr">

</xml_diff>

<commit_message>
WIP: cuadro de firma, combo de planta y backlog (recuperado)
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
@@ -5004,11 +5004,17 @@
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I51" s="11" t="n"/>
-      <c r="J51" s="20" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J51" s="20" t="inlineStr">
+        <is>
+          <t>Validado con la Product Owner (registrado el 27-09-2026 por indicación de Bryan Chávez).</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="27.6" customHeight="1" s="24">
       <c r="A52" s="11" t="inlineStr">
@@ -6310,11 +6316,17 @@
       </c>
       <c r="H80" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I80" s="11" t="n"/>
-      <c r="J80" s="20" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I80" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J80" s="20" t="inlineStr">
+        <is>
+          <t>Validado con la Product Owner (registrado el 27-09-2026 por indicación de Bryan Chávez).</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="27.6" customHeight="1" s="24">
       <c r="A81" s="11" t="inlineStr">

</xml_diff>